<commit_message>
Ajout du document synthétisant élargi
</commit_message>
<xml_diff>
--- a/Etude_sectorielle_Maroc.xlsx
+++ b/Etude_sectorielle_Maroc.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050" firstSheet="10" activeTab="13"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="7050"/>
   </bookViews>
   <sheets>
     <sheet name="Sommaire" sheetId="1" r:id="rId1"/>
@@ -2222,7 +2222,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B10" s="7" t="s">
         <v>12</v>
       </c>
@@ -2236,7 +2236,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="11" spans="2:5" ht="87" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
       <c r="B11" s="7" t="s">
         <v>12</v>
       </c>
@@ -2264,7 +2264,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="2:5" ht="72.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:5" ht="29" x14ac:dyDescent="0.35">
       <c r="B13" s="9" t="s">
         <v>21</v>
       </c>
@@ -2278,7 +2278,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="14" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="14" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B14" s="9" t="s">
         <v>21</v>
       </c>
@@ -2292,7 +2292,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="2:5" ht="43.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B15" s="9" t="s">
         <v>21</v>
       </c>
@@ -2306,7 +2306,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="16" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B16" s="9" t="s">
         <v>21</v>
       </c>
@@ -2320,7 +2320,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="2:5" ht="29" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B17" s="9" t="s">
         <v>21</v>
       </c>

</xml_diff>